<commit_message>
docs(workbook): mark Config and Segments as read by the importer (#5)
The sheet map on Readme and the sheet table in WORKBOOK_CONTRACT.md still
called Config and Segments "Input area defined; read by the data importer
(v0.2.0, not built)". The importer (#71) reads both: Config for the run
settings, Segments for the segment selection. Both rows now say so, and the
template is regenerated from the generator. The #5 audit asked for this
correction.

Validated: python tools/check.py passes all gates, including the template
regression suite (generator equality, contract tables).
Not validated: opening the template in Excel.
</commit_message>
<xml_diff>
--- a/src/workbook/IRRBB_Template.xlsx
+++ b/src/workbook/IRRBB_Template.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="195" uniqueCount="136">
   <si>
     <t xml:space="preserve">IRRBB Toolkit</t>
   </si>
@@ -131,13 +131,16 @@
     <t xml:space="preserve">User</t>
   </si>
   <si>
-    <t xml:space="preserve">Input area defined; read by the data importer (v0.2.0, not built)</t>
+    <t xml:space="preserve">Implemented: run settings read by the data importer (#71)</t>
   </si>
   <si>
     <t xml:space="preserve">Segments</t>
   </si>
   <si>
     <t xml:space="preserve">shSegments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implemented: segment selection read by the data importer (#71)</t>
   </si>
   <si>
     <t xml:space="preserve">DataSummary</t>
@@ -733,131 +736,131 @@
         <v>26</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C17" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -889,12 +892,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3">
@@ -902,18 +905,18 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="8"/>
     </row>
@@ -925,73 +928,73 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="D13" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="D13" s="4" t="s">
+      <c r="I13" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="J13" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="L13" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="N13" s="4" t="s">
         <v>127</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="K13" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1044,98 +1047,98 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -1170,51 +1173,51 @@
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7" s="5" t="s">
         <v>83</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -1265,12 +1268,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3">
@@ -1278,135 +1281,135 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B12" s="7"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="J13" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="L13" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="M13" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="N13" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="P13" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q13" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="S13" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="T13" s="4" t="s">
         <v>99</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="U13" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="E13" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="J13" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="L13" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="N13" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="P13" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q13" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="S13" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="T13" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="U13" s="4" t="s">
-        <v>99</v>
-      </c>
       <c r="V13" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="W13" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="X13" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="Y13" s="4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="Z13" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="AA13" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="AB13" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>
@@ -1437,12 +1440,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3">
@@ -1450,12 +1453,12 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1486,12 +1489,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="3">
@@ -1499,12 +1502,12 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1535,12 +1538,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3">
@@ -1548,12 +1551,12 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1584,12 +1587,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="3">
@@ -1597,12 +1600,12 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>
@@ -1633,12 +1636,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3">
@@ -1646,12 +1649,12 @@
         <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: name the project K-IRRBB
Use the project name K-IRRBB, as VBA-SACCR-Toolkit uses K-SACCR: the README
heading and purpose line, the headings of CONTRIBUTING, INSTALLATION,
RELEASING, SECURITY and CODE_OF_CONDUCT, the CHANGELOG, the PR template,
REPOSITORY_STRUCTURE, WORKBOOK_CONTRACT, VBA_HOUSE_STYLE, docs/assets, the
daily traffic alert text and the title on the workbook's Readme sheet. The
template IRRBB_Template.xlsx is regenerated from build_template.py.

The repository name VBA-IRRBB-Toolkit, its URLs, file names, identifiers and
the IRRBB_ prefix are unchanged; IRRBB as the subject (interest rate risk in
the banking book) is kept where it names the subject.

Validated: python tools/check.py --ci passes every gate on this commit;
build_template.py --check reports the template matches its source; the tool
unit tests pass (155, 7 skipped).
Not validated: the regenerated template was not opened in Excel; no Excel
compile or regression run.
</commit_message>
<xml_diff>
--- a/src/workbook/IRRBB_Template.xlsx
+++ b/src/workbook/IRRBB_Template.xlsx
@@ -61,12 +61,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="154">
   <si>
     <t xml:space="preserve">K-IRRBB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IRRBB Toolkit</t>
   </si>
   <si>
     <t xml:space="preserve">Start with Config and Segments. Import data in the development workbook, then review DataSummary. Yellow cells are inputs; blue tabs hold outputs.</t>
@@ -789,291 +786,291 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>4</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>6</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>10</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="C14" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="E14" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>30</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="C16" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="C17" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>38</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="C18" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="C19" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="C20" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>47</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="C21" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="9" t="s">
         <v>50</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="C22" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>53</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>63</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1132,115 +1129,115 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="H12" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="D13" s="11" t="s">
+      <c r="E13" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="F13" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="H13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="I13" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="J13" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="N13" s="11" t="s">
         <v>145</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -1309,104 +1306,104 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>82</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1451,62 +1448,62 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C6" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>96</v>
-      </c>
       <c r="C7" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1"/>
@@ -1573,161 +1570,161 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="L12" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="P12" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="P12" s="12" t="s">
+      <c r="S12" s="12" t="s">
         <v>113</v>
-      </c>
-      <c r="S12" s="12" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="D13" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="E13" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="G13" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="H13" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="I13" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="I13" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="J13" s="11" t="s">
+      <c r="N13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="P13" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q13" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="S13" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="T13" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="L13" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="P13" s="11" t="s">
+      <c r="U13" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="V13" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="Q13" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="U13" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="V13" s="11" t="s">
+      <c r="W13" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="W13" s="11" t="s">
+      <c r="X13" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="X13" s="11" t="s">
+      <c r="Y13" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="Y13" s="11" t="s">
+      <c r="Z13" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="Z13" s="11" t="s">
+      <c r="AA13" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="AA13" s="11" t="s">
+      <c r="AB13" s="11" t="s">
         <v>129</v>
-      </c>
-      <c r="AB13" s="11" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1783,24 +1780,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -1853,24 +1850,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -1923,24 +1920,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -1993,24 +1990,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -2063,24 +2060,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>

</xml_diff>

<commit_message>
docs: name the project K-IRRBB (#104)
Use the project name K-IRRBB, as VBA-SACCR-Toolkit uses K-SACCR: the README
heading and purpose line, the headings of CONTRIBUTING, INSTALLATION,
RELEASING, SECURITY and CODE_OF_CONDUCT, the CHANGELOG, the PR template,
REPOSITORY_STRUCTURE, WORKBOOK_CONTRACT, VBA_HOUSE_STYLE, docs/assets, the
daily traffic alert text and the title on the workbook's Readme sheet. The
template IRRBB_Template.xlsx is regenerated from build_template.py.

The repository name VBA-IRRBB-Toolkit, its URLs, file names, identifiers and
the IRRBB_ prefix are unchanged; IRRBB is kept where it names the subject.

Validated: python tools/check.py --ci passes every gate; build_template.py
--check reports the template matches its source; the tool unit tests pass
(155, 7 skipped).
Not validated: the regenerated template was not opened in Excel; no Excel
compile or regression run.
</commit_message>
<xml_diff>
--- a/src/workbook/IRRBB_Template.xlsx
+++ b/src/workbook/IRRBB_Template.xlsx
@@ -61,12 +61,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="154">
   <si>
     <t xml:space="preserve">K-IRRBB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IRRBB Toolkit</t>
   </si>
   <si>
     <t xml:space="preserve">Start with Config and Segments. Import data in the development workbook, then review DataSummary. Yellow cells are inputs; blue tabs hold outputs.</t>
@@ -789,291 +786,291 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>4</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>6</v>
-      </c>
-      <c r="B6" s="9" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" s="9" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
       <c r="A8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>10</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="C12" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="D12" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="E12" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="D13" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="14" ht="32" customHeight="1">
       <c r="A14" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="9" t="s">
+      <c r="C14" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="9" t="s">
+      <c r="E14" s="9" t="s">
         <v>27</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="9" t="s">
+      <c r="C15" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="9" t="s">
         <v>30</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>26</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B16" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="9" t="s">
+      <c r="C16" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="D16" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="E16" s="9" t="s">
         <v>35</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="C17" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>38</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
       <c r="A18" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="B18" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="9" t="s">
+      <c r="C18" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E18" s="9" t="s">
         <v>41</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="B19" s="9" t="s">
+      <c r="C19" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>44</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="B20" s="9" t="s">
+      <c r="C20" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>47</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="C21" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="9" t="s">
         <v>50</v>
-      </c>
-      <c r="C21" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
       <c r="A22" s="9" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="C22" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>53</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" ht="36" customHeight="1">
       <c r="A27" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B27" s="9" t="s">
         <v>57</v>
-      </c>
-      <c r="B27" s="9" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="28" ht="36" customHeight="1">
       <c r="A28" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>59</v>
-      </c>
-      <c r="B28" s="9" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="29" ht="36" customHeight="1">
       <c r="A29" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B29" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="B29" s="9" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="30" ht="36" customHeight="1">
       <c r="A30" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="9" t="s">
         <v>63</v>
-      </c>
-      <c r="B30" s="9" t="s">
-        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1132,115 +1129,115 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>137</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6" ht="36" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" ht="24" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" ht="36" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="H12" s="12" t="s">
         <v>143</v>
-      </c>
-      <c r="H12" s="12" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>145</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>146</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="D13" s="11" t="s">
+      <c r="E13" s="11" t="s">
         <v>147</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="F13" s="11" t="s">
         <v>148</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="H13" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="I13" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="J13" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="M13" s="11" t="s">
+        <v>153</v>
+      </c>
+      <c r="N13" s="11" t="s">
         <v>145</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>146</v>
       </c>
     </row>
   </sheetData>
@@ -1309,104 +1306,104 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" ht="34" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="5"/>
       <c r="C6" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="D6" s="9" t="s">
         <v>72</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="5"/>
       <c r="C7" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" ht="26" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B8" s="6"/>
       <c r="C8" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>77</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B9" s="6"/>
       <c r="C9" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B10" s="5"/>
       <c r="C10" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>82</v>
-      </c>
-      <c r="D10" s="9" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B11" s="5"/>
       <c r="C11" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="D11" s="9" t="s">
         <v>85</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
       <c r="A12" s="13" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1451,62 +1448,62 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" ht="38" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="10" customHeight="1"/>
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="B5" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="C5" s="4" t="s">
         <v>90</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C6" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>96</v>
-      </c>
       <c r="C7" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="B8" s="9" t="s">
-        <v>98</v>
-      </c>
       <c r="C8" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1"/>
@@ -1573,161 +1570,161 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B4" s="8"/>
     </row>
     <row r="5" ht="24" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B5" s="8"/>
     </row>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B6" s="7"/>
     </row>
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B7" s="7"/>
     </row>
     <row r="8" ht="24" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B8" s="7"/>
     </row>
     <row r="9" ht="24" customHeight="1">
       <c r="A9" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B9" s="7"/>
     </row>
     <row r="10" ht="24" customHeight="1">
       <c r="A10" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B10" s="7"/>
     </row>
     <row r="11" ht="36" customHeight="1">
       <c r="A11" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B11" s="7"/>
     </row>
     <row r="12" ht="36" customHeight="1">
       <c r="A12" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="G12" s="12" t="s">
+      <c r="L12" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="L12" s="12" t="s">
+      <c r="P12" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="P12" s="12" t="s">
+      <c r="S12" s="12" t="s">
         <v>113</v>
-      </c>
-      <c r="S12" s="12" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="13" ht="42" customHeight="1">
       <c r="A13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="D13" s="11" t="s">
         <v>117</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="E13" s="11" t="s">
         <v>118</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="G13" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="H13" s="11" t="s">
         <v>120</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="I13" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="J13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="I13" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="J13" s="11" t="s">
+      <c r="N13" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="P13" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="Q13" s="11" t="s">
+        <v>67</v>
+      </c>
+      <c r="S13" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="T13" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="L13" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="P13" s="11" t="s">
+      <c r="U13" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="V13" s="11" t="s">
         <v>123</v>
       </c>
-      <c r="Q13" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="S13" s="11" t="s">
-        <v>77</v>
-      </c>
-      <c r="T13" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="U13" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="V13" s="11" t="s">
+      <c r="W13" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="W13" s="11" t="s">
+      <c r="X13" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="X13" s="11" t="s">
+      <c r="Y13" s="11" t="s">
         <v>126</v>
       </c>
-      <c r="Y13" s="11" t="s">
+      <c r="Z13" s="11" t="s">
         <v>127</v>
       </c>
-      <c r="Z13" s="11" t="s">
+      <c r="AA13" s="11" t="s">
         <v>128</v>
       </c>
-      <c r="AA13" s="11" t="s">
+      <c r="AB13" s="11" t="s">
         <v>129</v>
-      </c>
-      <c r="AB13" s="11" t="s">
-        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -1783,24 +1780,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -1853,24 +1850,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -1923,24 +1920,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -1993,24 +1990,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>
@@ -2063,24 +2060,24 @@
     </row>
     <row r="2" ht="27" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="4" ht="24" customHeight="1"/>
     <row r="5" ht="26" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1"/>

</xml_diff>